<commit_message>
feat: integrate real templates — 38 copywritings + 27 image pairs + DM/reply variations + 37/50 keywords + synonym engine
</commit_message>
<xml_diff>
--- a/materials/materials.xlsx
+++ b/materials/materials.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,12 +457,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>效果展示</t>
+          <t>喜悦分享</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>用了这个方法，白斑真的淡了！前后对比太明显了</t>
+          <t>遇到高兴的事很难不分享出来。</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -485,12 +485,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>经验分享</t>
+          <t>喜悦分享</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>我也是白斑困扰多年，终于找到了方法</t>
+          <t>遇到高兴的事真的忍不住想要分享出来。</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -513,23 +513,1003 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>互动引导</t>
+          <t>庆祝</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>有同样困扰的姐妹看过来，这个方法真的有用</t>
+          <t>今年最最最值得庆祝的喜悦，分享给大家。</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>上岸</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>真的会有人恭喜我吗，成功上岸啦</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>20</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>上岸</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>这是26年最值得炫耀的一件事，真的会有人恭喜我吗</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>分享</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>和素未谋面的陌生朋友分享分享我的高兴事</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>上岸</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>真的会有人替我高兴吗，我也是成功上岸啦</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>20</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>分享</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>生活中的一份小美好，迫不及待地来跟大家一起分享</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>10</v>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="E9" t="n">
+        <v>15</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>上岸</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>幸福来得太突然了，终于让我在2026年上岸成功啦。</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>20</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>分享</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>这是我今年最值得分享的好事</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>15</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>康复</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>我就知道人不可能倒霉一辈子的，终于康复啦</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>20</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>康复</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>今年能拿得出手的一件事，白癜风终于好啦!大家可以夸夸我嘛</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>纪念</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>这是今年最有纪念意义的事儿，分享分享给大家，可以祝贺我吗</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>15</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>幸运</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>最近遇到的一份小幸运，可以得到大家的祝福吗</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>报喜</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>来跟朋友们报个喜，分享一件特别值得庆贺的事儿</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>15</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>骄傲</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>这也是今年最值得骄傲的一件事，快来恭喜恭喜我吧</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>上岸</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>没想到我也能上岸成功，可以得到陌生朋友的一句祝福吗</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>20</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>开心</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>哈哈哈我的开心事，忍不住想分享给陌生的朋友</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>15</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>礼物</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>这真的是我收到的最好最棒的一个礼物了，可以恭喜恭喜我吗</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>10</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>礼物</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>这真的是孩子收到的最好最棒的礼物了，开心了好久</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>10</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>上岸</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>幸福来得太突然了，历经几年，终于上岸了</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>20</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>康复</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>以后再也不用遮遮掩掩的了，被歧视的日子终于过去了</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>20</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>分享</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>美好的事想和大家分享</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>15</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>康复</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>再也不会被孤立了，终于好了</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>康复</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>终于恢复了，陌生的朋友能祝福祝福吗</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>20</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>幸福</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>幸福的事当然也要分享出来</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>15</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>康复</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>生活又给了我一次惊喜，嘿嘿终于康复了</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>20</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>期待</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>我也来分享分享我今年期待已久的喜事</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>15</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>期盼</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>我也来分享一件期盼许久的开心事</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>15</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>开心</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>我也来说说我盼了好久的开心事</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>15</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>分享</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>我也分享一下我心心念念的开心事</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>15</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>期待</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>我也来讲讲我期待了很久的开心事</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>15</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>大喜事</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>我也来和大家说说，今年我满心期盼的大喜事</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>15</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>好消息</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>我也来分享一下，今年我盼了好久的好消息</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>15</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>大喜事</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>我也来讲讲，今年我期待了许久的大喜事。</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>15</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>分享</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>我也来跟大家分享，今年我心心念念的大好事</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>15</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>康复</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>生活不会一帆风顺的，但是值得庆幸的是，终于康复啦</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>20</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>心愿</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>我也算是在今年了却了心愿了，陌生的朋友可以祝福祝福我吗</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>15</v>
+      </c>
+      <c r="F39" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -546,7 +1526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -592,26 +1572,26 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>手部对比</t>
+          <t>对比组 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>images/before_hand.jpg</t>
+          <t>images/1-(1)_01.jpg</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>images/after_hand.jpg</t>
+          <t>images/1-(1)_02.jpg</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>手部</t>
+          <t>对比</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -625,26 +1605,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>面部对比</t>
+          <t>对比组 2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>images/before_face.jpg</t>
+          <t>images/1-(2)_01.jpg</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>images/after_face.jpg</t>
+          <t>images/1-(2)_02.jpg</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>面部</t>
+          <t>对比</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -658,28 +1638,820 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>腿部对比</t>
+          <t>对比组 3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>images/before_leg.jpg</t>
+          <t>images/1-(3)_01.jpg</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>images/after_leg.jpg</t>
+          <t>images/1-(3)_02.jpg</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>腿部</t>
+          <t>对比</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>10</v>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>对比组 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>images/1-(4)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>images/1-(4)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>对比组 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>images/1-(5)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>images/1-(5)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>对比组 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>images/1-(6)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>images/1-(6)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>10</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>对比组 7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>images/1-(7)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>images/1-(7)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>对比组 8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>images/1-(8)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>images/1-(8)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>对比组 9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>images/1-(9)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>images/1-(9)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>对比组 10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>images/1-(10)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>images/1-(10)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>10</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>对比组 11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>images/1-(11)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>images/1-(11)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>对比组 12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>images/1-(12)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>images/1-(12)_03.png</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>10</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>对比组 13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>images/1-(13)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>images/1-(13)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>对比组 14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>images/1-(14)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>images/1-(14)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>对比组 15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>images/1-(15)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>images/1-(15)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>对比组 16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>images/1-(16)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>images/1-(16)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>10</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>对比组 17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>images/1-(17)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>images/1-(17)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>对比组 18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>images/1-(18)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>images/1-(18)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>10</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>对比组 19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>images/1-(19)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>images/1-(19)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>10</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>对比组 20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>images/1-(20)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>images/1-(20)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>10</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>对比组 21</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>images/1-(21)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>images/1-(21)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>对比组 22</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>images/1-(22)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>images/1-(22)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>10</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>对比组 23</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>images/1-(23)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>images/1-(23)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>10</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>对比组 24</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>images/1-(24)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>images/1-(24)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>10</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>对比组 25</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>images/1-(25)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>images/1-(25)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>10</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>对比组 26</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>images/1-(26)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>images/1-(26)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>10</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>对比组 27</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>images/1-(27)_01.jpg</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>images/1-(27)_02.jpg</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>对比</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>10</v>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -696,7 +2468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -732,7 +2504,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>看到你评论问我，我是吃药加照光弄好的</t>
+          <t>看你评论问我，我是吃药加光照弄好的</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -747,15 +2519,115 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>默认变体</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>看到你的评论了，我用的是吃药配合光疗，现在已经好了</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>默认变体</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>刚看到你的评论，我是坚持吃药加光照治疗恢复的</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>默认变体</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>你好呀，看你在评论区问我，我是吃药+光疗治好的</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>追问</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>具体就是口服药+定期照光，坚持了半年左右，你可以试试</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>具体就是每天按时吃药，定期去医院照光，坚持了大半年就好了</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>追问</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>方法就是口服药搭配光照治疗，一定要坚持才有效果</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>关心</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>你可以先了解一下光疗，我是过来人，有什么不懂的可以问我</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -772,7 +2644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,7 +2680,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>怎么治,如何治,什么方法</t>
+          <t>怎么治,如何治,什么方法,怎么弄,怎么好</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -818,7 +2690,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>吃药加照光</t>
+          <t>这个是我用光照加吃药好的</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -833,7 +2705,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>真的吗,有用吗,效果</t>
+          <t>怎么治,如何治,什么方法,怎么弄,怎么好</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -843,7 +2715,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>真的！坚持就会有效果</t>
+          <t>我是吃药配合光疗恢复的，坚持最重要</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -858,20 +2730,195 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>怎么治,如何治,什么方法,怎么弄,怎么好</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>就是坚持吃药加照光，慢慢就好了</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>真的吗,有用吗,效果,真有效,管用</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>真的有用！我坚持了半年多，变化特别明显</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>真的吗,有用吗,效果,真有效,管用</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>当然是真的！你看我恢复的效果就知道了</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>多久,多长时间,几年,几个月</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>我坚持了大半年，每个人的情况不一样，但坚持就会有效果</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>哪里治,什么医院,哪个医生,推荐</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>我就是在当地医院看的，关键是坚持吃药和照光</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>恭喜,祝福,真好,太好了,羡慕</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>emoji</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>😊🙏❤️</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>加油,会好的,接好运,沾沾</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>emoji</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>💪✨🍀</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>*</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>emoji</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>😊👍</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>😊👍🌹</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>